<commit_message>
Årsplan: OPO er fastlagt til uge 4, 5 og 6
Noten nederst sagde, at ugenumrene ikke var fastlagt. Den står nu som OPO i
9. klasse med uge 4, 5 og 6, og at planen revideres når vi nærmer os.

Rettet både på siden og i regnearkets Projektopgave-ark, så de siger det samme.
Efterset at regnearket er uændret bortset fra de to celler: samme tre ark,
samme dimensioner, kolonnebredder og flettede celler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VgEVctXq3tNeZxt6iAFBPu
</commit_message>
<xml_diff>
--- a/aarsplan-matematik-2026-27.xlsx
+++ b/aarsplan-matematik-2026-27.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Årsplan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overblik" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projektopgave" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Årsplan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overblik" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Projektopgave" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Årsplan'!$4:$4</definedName>
@@ -701,7 +701,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="28">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -1595,7 +1594,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="45" t="inlineStr">
         <is>
@@ -1688,8 +1686,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="28">
       <c r="A11" s="50" t="inlineStr">
         <is>
@@ -1769,8 +1765,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="28">
       <c r="A20" s="50" t="inlineStr">
         <is>
@@ -1832,14 +1826,14 @@
     <row r="1" ht="17.35" customHeight="1" s="28">
       <c r="A1" s="44" t="inlineStr">
         <is>
-          <t>Projektopgaven i 9. klasse · plads til datoer</t>
+          <t>OPO i 9. klasse · uge 4, 5 og 6</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="28">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Ugenumrene herunder er ikke fastlagt endnu. Skriv dem ind, når skolens plan ligger fast — så flytter jeg forløbene i årsplanen, hvis de kolliderer.</t>
+          <t>Ugenumrene er fastlagt til 4, 5 og 6. Plan revideres når vi nærmer os.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ret regnearkets indledning, så den følger den flyttede plan
Vinterferien er bekræftet til kun uge 7, hvilket planen allerede var lagt
efter. Men regnearkets indledning i celle A2 sagde stadig uge 33 til uge 6 og
at repetitionen begyndte i uge 8 — den blev kun rettet på siden.

Efterset at side og regneark nu er enige: samme ugerækkefølge, og samme
beskrivelse af hvor OPO, vinterferie og repetition ligger.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VgEVctXq3tNeZxt6iAFBPu
</commit_message>
<xml_diff>
--- a/aarsplan-matematik-2026-27.xlsx
+++ b/aarsplan-matematik-2026-27.xlsx
@@ -697,7 +697,7 @@
     <row r="2" ht="15" customHeight="1" s="28">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Kernestoffet er fordelt på uge 33 til uge 6, så alle forløb er kørt igennem inden vinterferien. Uge 8 og frem er sat af til repetition og prøvetræning.</t>
+          <t>Kernestoffet er fordelt på uge 33 til uge 10. Uge 4 til 6 er OPO, og uge 7 er vinterferie, så de tre sidste geometriforløb ligger i uge 8, 9 og 10. Uge 11 og frem er sat af til repetition og prøvetræning.</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
           <t>Mål på flader</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>Bestemme areal og omkreds af komplekse figurer med digitale værktøjer
 Dele en kompleks figur op i kendte figurer
@@ -1542,7 +1542,7 @@
           <t>Rumfang og vægt</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>Beregne rumfanget af bl.a. keglestubbe og pyramidestubbe
 Bestemme massefylde, vægt og rumfang af genstande fra hverdagen</t>

</xml_diff>